<commit_message>
Planilla de compras actualizada, hojas de datos
</commit_message>
<xml_diff>
--- a/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
+++ b/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
-  <si>
-    <t xml:space="preserve">PCB</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="47">
+  <si>
+    <t xml:space="preserve">PCB (LDO)</t>
   </si>
   <si>
     <t xml:space="preserve">Gabinete</t>
@@ -31,6 +31,9 @@
     <t xml:space="preserve">Componente</t>
   </si>
   <si>
+    <t xml:space="preserve">Detalle</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cantidad</t>
   </si>
   <si>
@@ -40,7 +43,115 @@
     <t xml:space="preserve">Datasheet</t>
   </si>
   <si>
+    <t xml:space="preserve">Encapsulado</t>
+  </si>
+  <si>
     <t xml:space="preserve">Proveedor</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Pines 2x1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V_Rs_test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V_current_test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V_voltage_test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V_ref_test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V_ref_c_test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transistor npn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2N3904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transistor pnp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2N3906</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transistor PMOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRF4905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC547</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC557</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.7k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.4k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.8k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.7k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alambre Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencia Prog.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TL431LP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amplificador Op.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LM358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDIP-8</t>
   </si>
   <si>
     <t xml:space="preserve">Total PCB</t>
@@ -56,14 +167,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -82,6 +195,12 @@
     </font>
     <font>
       <u val="single"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -147,16 +266,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -164,7 +303,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -245,117 +396,611 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13.47"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="G1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="L1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="F2" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="0" t="s">
+      <c r="M2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="N2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="O2" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="P2" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="A3" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="str">
+        <f aca="false">HYPERLINK("Datasheets/2N3904.PDF","Ver datasheet")</f>
+        <v>Ver datasheet</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7" t="str">
+        <f aca="false">HYPERLINK("Datasheets/2N3906.PDF","Ver datasheet")</f>
+        <v>Ver datasheet</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="str">
+        <f aca="false">HYPERLINK("Datasheets/IRF4905.pdf","Ver datasheet")</f>
+        <v>Ver datasheet</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
+      <c r="A13" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="0" t="n">
-        <f aca="false">SUM(C3:C12)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" s="0" t="n">
-        <f aca="false">SUM(I3:I12)</f>
-        <v>0</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
+      <c r="A15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="0" t="n">
-        <f aca="false">SUM(B14,H14)</f>
-        <v>0</v>
-      </c>
+      <c r="D16" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="3"/>
+      <c r="A17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L18" s="0"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="8"/>
+      <c r="F19" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1"/>
+      <c r="F22" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="1"/>
+      <c r="F23" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="0" t="str">
+        <f aca="false">HYPERLINK("Datasheets/TL431.PDF","Ver datasheet")</f>
+        <v>Ver datasheet</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="8" t="str">
+        <f aca="false">HYPERLINK("Datasheets/LM358.PDF","Ver datasheet")</f>
+        <v>Ver datasheet</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="L25" s="0"/>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="10"/>
+      <c r="L26" s="0"/>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="0"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="0"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="0"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C31" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" s="11" t="n">
+        <f aca="false">SUM( PRODUCT(C3,D3),PRODUCT(C4,D4),PRODUCT(C5,D5),PRODUCT(C6,D6), PRODUCT(C7,D7),PRODUCT(C8,D8),PRODUCT(C9,D9),PRODUCT(C10,D10), PRODUCT(C11,D11),PRODUCT(C12,D12),PRODUCT(C13,D13),PRODUCT(C14,D14), PRODUCT(C15,D15),PRODUCT(C16,D16),PRODUCT(C17,D17),PRODUCT(C18,D18), PRODUCT(C19,D19),PRODUCT(C20,D20),PRODUCT(C21,D21),PRODUCT(C22,D22), PRODUCT(C23,D23),PRODUCT(C24,D24),PRODUCT(C25,D25),PRODUCT(C26,D26), PRODUCT(C27,D27),PRODUCT(C28,D28),PRODUCT(C29,D29),PRODUCT(C30,D30), PRODUCT(C31,D31),PRODUCT(C32,D32),PRODUCT(C33,D33) )</f>
+        <v>0</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="M35" s="1" t="n">
+        <f aca="false">SUM(N3:N12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+      <c r="L36" s="12"/>
+      <c r="M36" s="12"/>
+      <c r="N36" s="12"/>
+      <c r="O36" s="12"/>
+      <c r="P36" s="12"/>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <f aca="false">SUM(B35,M35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Agrupación de modulos en diseño de PCB
</commit_message>
<xml_diff>
--- a/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
+++ b/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
@@ -148,7 +148,7 @@
     <t xml:space="preserve">Amplificador Op.</t>
   </si>
   <si>
-    <t xml:space="preserve">LM358</t>
+    <t xml:space="preserve">LM324</t>
   </si>
   <si>
     <t xml:space="preserve">PDIP-8</t>
@@ -167,11 +167,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -199,11 +198,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -266,7 +260,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -279,7 +273,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -291,27 +285,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -399,12 +381,12 @@
   <dimension ref="A1:P38"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13.47"/>
   </cols>
   <sheetData>
@@ -430,7 +412,7 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -442,7 +424,7 @@
       <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -465,107 +447,101 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1"/>
+      <c r="C3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="L3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="1"/>
+      <c r="C4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1"/>
+      <c r="C5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1"/>
+      <c r="C6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1"/>
+      <c r="C7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1"/>
+      <c r="C8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="1" t="str">
@@ -580,16 +556,16 @@
       <c r="A10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="7" t="str">
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6" t="str">
         <f aca="false">HYPERLINK("Datasheets/2N3906.PDF","Ver datasheet")</f>
         <v>Ver datasheet</v>
       </c>
@@ -598,16 +574,16 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="0" t="n">
+      <c r="C11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="1" t="str">
@@ -619,166 +595,157 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="8"/>
+      <c r="D12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5"/>
       <c r="F12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="0" t="n">
+      <c r="C13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="0" t="n">
+      <c r="C14" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="9" t="s">
+      <c r="D14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="0" t="n">
+      <c r="C15" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D15" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="9" t="s">
+      <c r="D15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="0" t="n">
+      <c r="C16" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D16" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="s">
+      <c r="D16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="9" t="s">
+      <c r="C17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="0" t="n">
+      <c r="C18" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="9" t="s">
+      <c r="D18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="8"/>
-      <c r="F19" s="9" t="s">
+      <c r="C19" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5"/>
+      <c r="F19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L19" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="9" t="s">
+      <c r="C20" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -786,17 +753,16 @@
       <c r="A21" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="9" t="s">
+      <c r="C21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -804,121 +770,114 @@
       <c r="A22" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="9" t="s">
+      <c r="C22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>28</v>
       </c>
+      <c r="I22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="9" t="s">
+      <c r="C23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="0" t="str">
+      <c r="C24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="1" t="str">
         <f aca="false">HYPERLINK("Datasheets/TL431.PDF","Ver datasheet")</f>
         <v>Ver datasheet</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L24" s="0"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="0" t="n">
+      <c r="C25" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="8" t="str">
-        <f aca="false">HYPERLINK("Datasheets/LM358.PDF","Ver datasheet")</f>
+      <c r="D25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="str">
+        <f aca="false">HYPERLINK("Datasheets/LM324.PDF","Ver datasheet")</f>
         <v>Ver datasheet</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="F25" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L25" s="0"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="10"/>
-      <c r="L26" s="0"/>
+      <c r="C26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="0"/>
+      <c r="C27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="0"/>
+      <c r="C28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="0"/>
+      <c r="C29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="0" t="n">
+      <c r="C30" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="1" t="n">
@@ -926,7 +885,7 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="0" t="n">
+      <c r="C31" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="1" t="n">
@@ -934,7 +893,7 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="0" t="n">
+      <c r="C32" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="1" t="n">
@@ -942,7 +901,7 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="0" t="n">
+      <c r="C33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="1" t="n">
@@ -965,7 +924,7 @@
       <c r="A35" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="1" t="n">
         <f aca="false">SUM( PRODUCT(C3,D3),PRODUCT(C4,D4),PRODUCT(C5,D5),PRODUCT(C6,D6), PRODUCT(C7,D7),PRODUCT(C8,D8),PRODUCT(C9,D9),PRODUCT(C10,D10), PRODUCT(C11,D11),PRODUCT(C12,D12),PRODUCT(C13,D13),PRODUCT(C14,D14), PRODUCT(C15,D15),PRODUCT(C16,D16),PRODUCT(C17,D17),PRODUCT(C18,D18), PRODUCT(C19,D19),PRODUCT(C20,D20),PRODUCT(C21,D21),PRODUCT(C22,D22), PRODUCT(C23,D23),PRODUCT(C24,D24),PRODUCT(C25,D25),PRODUCT(C26,D26), PRODUCT(C27,D27),PRODUCT(C28,D28),PRODUCT(C29,D29),PRODUCT(C30,D30), PRODUCT(C31,D31),PRODUCT(C32,D32),PRODUCT(C33,D33) )</f>
         <v>0</v>
       </c>
@@ -978,17 +937,17 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="L36" s="12"/>
-      <c r="M36" s="12"/>
-      <c r="N36" s="12"/>
-      <c r="O36" s="12"/>
-      <c r="P36" s="12"/>
+      <c r="A36" s="9"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">

</xml_diff>

<commit_message>
Diseño PCB :  Test con gnd en comun
</commit_message>
<xml_diff>
--- a/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
+++ b/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="53">
   <si>
     <t xml:space="preserve">PCB (LDO)</t>
   </si>
@@ -157,13 +157,19 @@
     <t xml:space="preserve">PDIP-8</t>
   </si>
   <si>
+    <t xml:space="preserve">Disipador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ide-shop.com.ar/productos/disipador-to220-negro-aleteado-15x10x20mm-x5u/</t>
+  </si>
+  <si>
     <t xml:space="preserve">PCB virgen</t>
   </si>
   <si>
     <t xml:space="preserve">10x10 doble faz</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.ide-shop.com.ar/</t>
+    <t xml:space="preserve">https://www.ide-shop.com.ar/productos/placa-virgen-fr4-doble-faz/</t>
   </si>
   <si>
     <t xml:space="preserve">Total PCB</t>
@@ -949,28 +955,37 @@
       <c r="A26" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="C26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>866</v>
+      </c>
+      <c r="E26" s="6"/>
+      <c r="F26" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G26" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="1" t="n">
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="1" t="n">
         <v>3798</v>
       </c>
-      <c r="E26" s="6"/>
-      <c r="G26" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="E27" s="6"/>
+      <c r="G27" s="5" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="1" t="n">
@@ -1034,14 +1049,14 @@
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B35" s="1" t="n">
         <f aca="false">SUM( PRODUCT(C3,D3),PRODUCT(C4,D4),PRODUCT(C5,D5),PRODUCT(C6,D6), PRODUCT(C7,D7),PRODUCT(C8,D8),PRODUCT(C9,D9),PRODUCT(C10,D10), PRODUCT(C11,D11),PRODUCT(C12,D12),PRODUCT(C13,D13),PRODUCT(C14,D14), PRODUCT(C15,D15),PRODUCT(C16,D16),PRODUCT(C17,D17),PRODUCT(C18,D18), PRODUCT(C19,D19),PRODUCT(C20,D20),PRODUCT(C21,D21),PRODUCT(C22,D22), PRODUCT(C23,D23),PRODUCT(C24,D24),PRODUCT(C25,D25),PRODUCT(C26,D26), PRODUCT(C27,D27),PRODUCT(C28,D28),PRODUCT(C29,D29),PRODUCT(C30,D30), PRODUCT(C31,D31),PRODUCT(C32,D32),PRODUCT(C33,D33) )</f>
-        <v>18610</v>
+        <v>23274</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="M35" s="1" t="n">
         <f aca="false">SUM(N3:N12)</f>
@@ -1063,11 +1078,11 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B37" s="1" t="n">
         <f aca="false">SUM(B35,M35)</f>
-        <v>18610</v>
+        <v>23274</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1080,6 +1095,8 @@
     <hyperlink ref="G11" r:id="rId3" display="https://www.microelectronicash.com"/>
     <hyperlink ref="G12" r:id="rId4" display="https://www.microelectronicash.com"/>
     <hyperlink ref="G13" r:id="rId5" display="https://www.microelectronicash.com"/>
+    <hyperlink ref="G26" r:id="rId6" display="https://www.ide-shop.com.ar/productos/disipador-to220-negro-aleteado-15x10x20mm-x5u/"/>
+    <hyperlink ref="G27" r:id="rId7" display="https://www.ide-shop.com.ar/productos/placa-virgen-fr4-doble-faz/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Etiquetas checkpoints, facturas y presupuesto
</commit_message>
<xml_diff>
--- a/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
+++ b/Documentación/Hoja de Calculo- Presupuesto/Presupuesto.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="54">
   <si>
     <t xml:space="preserve">PCB (LDO)</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t xml:space="preserve">1.7k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preset ajust</t>
   </si>
   <si>
     <t xml:space="preserve">Alambre Resistor</t>
@@ -290,7 +293,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -329,10 +332,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -512,7 +511,7 @@
       <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="7" t="n">
         <v>180</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -529,7 +528,7 @@
       <c r="C5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="7" t="n">
         <v>180</v>
       </c>
       <c r="G5" s="1" t="s">
@@ -546,7 +545,7 @@
       <c r="C6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="7" t="n">
         <v>180</v>
       </c>
       <c r="G6" s="1" t="s">
@@ -563,7 +562,7 @@
       <c r="C7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="7" t="n">
         <v>180</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -580,7 +579,7 @@
       <c r="C8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="7" t="n">
         <v>180</v>
       </c>
       <c r="G8" s="1" t="s">
@@ -598,7 +597,7 @@
         <v>9</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>350</v>
+        <v>246</v>
       </c>
       <c r="E9" s="1" t="str">
         <f aca="false">HYPERLINK("Datasheets/2N3904.PDF","Ver datasheet")</f>
@@ -622,7 +621,7 @@
         <v>5</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>350</v>
+        <v>203</v>
       </c>
       <c r="E10" s="7" t="str">
         <f aca="false">HYPERLINK("Datasheets/2N3906.PDF","Ver datasheet")</f>
@@ -643,10 +642,10 @@
         <v>23</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>3800</v>
+        <v>5352</v>
       </c>
       <c r="E11" s="1" t="str">
         <f aca="false">HYPERLINK("Datasheets/IRF4905.pdf","Ver datasheet")</f>
@@ -669,8 +668,8 @@
       <c r="C12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="1" t="n">
-        <v>350</v>
+      <c r="D12" s="8" t="n">
+        <v>246</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="7" t="s">
@@ -690,8 +689,8 @@
       <c r="C13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="1" t="n">
-        <v>350</v>
+      <c r="D13" s="8" t="n">
+        <v>203</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>19</v>
@@ -730,7 +729,7 @@
       <c r="C15" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="7" t="n">
         <v>75</v>
       </c>
       <c r="F15" s="9" t="s">
@@ -750,7 +749,7 @@
       <c r="C16" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="7" t="n">
         <v>75</v>
       </c>
       <c r="F16" s="9" t="s">
@@ -770,7 +769,7 @@
       <c r="C17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="7" t="n">
         <v>75</v>
       </c>
       <c r="F17" s="9" t="s">
@@ -790,7 +789,7 @@
       <c r="C18" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="7" t="n">
         <v>75</v>
       </c>
       <c r="F18" s="9" t="s">
@@ -810,7 +809,7 @@
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="7" t="n">
         <v>75</v>
       </c>
       <c r="E19" s="6"/>
@@ -831,7 +830,7 @@
       <c r="C20" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="7" t="n">
         <v>75</v>
       </c>
       <c r="F20" s="9" t="s">
@@ -851,7 +850,7 @@
       <c r="C21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="7" t="n">
         <v>75</v>
       </c>
       <c r="F21" s="9" t="s">
@@ -871,7 +870,7 @@
       <c r="C22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="7" t="n">
         <v>75</v>
       </c>
       <c r="F22" s="9" t="s">
@@ -883,116 +882,125 @@
       <c r="I22" s="7"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <v>3115</v>
+      </c>
+      <c r="E23" s="0"/>
+      <c r="F23" s="0"/>
+      <c r="G23" s="0"/>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="8" t="n">
+      <c r="B24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="n">
         <v>75</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F24" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="1" t="s">
+      <c r="G24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I24" s="6"/>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="1" t="n">
+      <c r="B25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="1" t="n">
         <v>2000</v>
       </c>
-      <c r="E24" s="1" t="str">
+      <c r="E25" s="1" t="str">
         <f aca="false">HYPERLINK("Datasheets/TL431.PDF","Ver datasheet")</f>
         <v>Ver datasheet</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" s="1" t="s">
+      <c r="G25" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>3480</v>
-      </c>
-      <c r="E25" s="6" t="str">
+      <c r="B26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>942</v>
+      </c>
+      <c r="E26" s="6" t="str">
         <f aca="false">HYPERLINK("Datasheets/LM324.PDF","Ver datasheet")</f>
         <v>Ver datasheet</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="1" t="n">
-        <v>866</v>
-      </c>
-      <c r="E26" s="6"/>
-      <c r="F26" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>46</v>
+      <c r="G26" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>866</v>
+      </c>
+      <c r="E27" s="6"/>
+      <c r="F27" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="1" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="1" t="n">
+      <c r="B28" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="1" t="n">
         <v>3798</v>
       </c>
-      <c r="E27" s="6"/>
-      <c r="G27" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>0</v>
+      <c r="E28" s="6"/>
+      <c r="G28" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1002,6 +1010,7 @@
       <c r="D29" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="E29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C30" s="1" t="n">
@@ -1049,14 +1058,14 @@
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B35" s="1" t="n">
-        <f aca="false">SUM( PRODUCT(C3,D3),PRODUCT(C4,D4),PRODUCT(C5,D5),PRODUCT(C6,D6), PRODUCT(C7,D7),PRODUCT(C8,D8),PRODUCT(C9,D9),PRODUCT(C10,D10), PRODUCT(C11,D11),PRODUCT(C12,D12),PRODUCT(C13,D13),PRODUCT(C14,D14), PRODUCT(C15,D15),PRODUCT(C16,D16),PRODUCT(C17,D17),PRODUCT(C18,D18), PRODUCT(C19,D19),PRODUCT(C20,D20),PRODUCT(C21,D21),PRODUCT(C22,D22), PRODUCT(C23,D23),PRODUCT(C24,D24),PRODUCT(C25,D25),PRODUCT(C26,D26), PRODUCT(C27,D27),PRODUCT(C28,D28),PRODUCT(C29,D29),PRODUCT(C30,D30), PRODUCT(C31,D31),PRODUCT(C32,D32),PRODUCT(C33,D33) )</f>
-        <v>23274</v>
+        <f aca="false">SUM( PRODUCT(C3,D3),PRODUCT(C4,D4),PRODUCT(C5,D5),PRODUCT(C6,D6), PRODUCT(C7,D7),PRODUCT(C8,D8),PRODUCT(C9,D9),PRODUCT(C10,D10), PRODUCT(C11,D11),PRODUCT(C12,D12),PRODUCT(C13,D13),PRODUCT(C14,D14), PRODUCT(C15,D15),PRODUCT(C16,D16),PRODUCT(C17,D17),PRODUCT(C18,D18), PRODUCT(C19,D19),PRODUCT(C20,D20),PRODUCT(C21,D21),PRODUCT(C22,D22), PRODUCT(C24,D24),PRODUCT(C25,D25),PRODUCT(C26,D26),PRODUCT(C27,D27), PRODUCT(C28,D28),PRODUCT(C28,D28),PRODUCT(C29,D29),PRODUCT(C30,D30), PRODUCT(C31,D31),PRODUCT(C32,D32),PRODUCT(C33,D33) )</f>
+        <v>27133</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M35" s="1" t="n">
         <f aca="false">SUM(N3:N12)</f>
@@ -1064,25 +1073,25 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="N36" s="11"/>
-      <c r="O36" s="11"/>
-      <c r="P36" s="11"/>
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="10"/>
+      <c r="N36" s="10"/>
+      <c r="O36" s="10"/>
+      <c r="P36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B37" s="1" t="n">
         <f aca="false">SUM(B35,M35)</f>
-        <v>23274</v>
+        <v>27133</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1095,8 +1104,8 @@
     <hyperlink ref="G11" r:id="rId3" display="https://www.microelectronicash.com"/>
     <hyperlink ref="G12" r:id="rId4" display="https://www.microelectronicash.com"/>
     <hyperlink ref="G13" r:id="rId5" display="https://www.microelectronicash.com"/>
-    <hyperlink ref="G26" r:id="rId6" display="https://www.ide-shop.com.ar/productos/disipador-to220-negro-aleteado-15x10x20mm-x5u/"/>
-    <hyperlink ref="G27" r:id="rId7" display="https://www.ide-shop.com.ar/productos/placa-virgen-fr4-doble-faz/"/>
+    <hyperlink ref="G27" r:id="rId6" display="https://www.ide-shop.com.ar/productos/disipador-to220-negro-aleteado-15x10x20mm-x5u/"/>
+    <hyperlink ref="G28" r:id="rId7" display="https://www.ide-shop.com.ar/productos/placa-virgen-fr4-doble-faz/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>